<commit_message>
validation stage business rules updated
</commit_message>
<xml_diff>
--- a/uploads_templates/uploads_for_validation/10.warehouse_capacity.xlsx
+++ b/uploads_templates/uploads_for_validation/10.warehouse_capacity.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Claude\Moove\RCCP\uploads_templates\uploads_for_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D70880-5BEF-4164-8C7D-929CD76ED58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7680A8BC-1D57-45F5-8544-67413288B8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11220" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17580" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="25">
   <si>
     <t>Warehouse code (e.g. UKP1, UKP3, UKP4, UKP5). Must exist in the masterdata.</t>
   </si>
@@ -50,6 +50,9 @@
     <t>60L</t>
   </si>
   <si>
+    <t>UKP3</t>
+  </si>
+  <si>
     <t>RCCP One — Warehouse Capacity Template</t>
   </si>
   <si>
@@ -87,6 +90,12 @@
   </si>
   <si>
     <t>BARREL</t>
+  </si>
+  <si>
+    <t>UKP4</t>
+  </si>
+  <si>
+    <t>UKP5</t>
   </si>
 </sst>
 </file>
@@ -106,35 +115,30 @@
       <sz val="9"/>
       <color rgb="FF7A5700"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF444444"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF444444"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -189,10 +193,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -503,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
@@ -532,35 +536,134 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="7">
         <v>4700</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="7">
         <v>365</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="3">
+      <c r="B5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="7">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="7">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="7">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="7">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="7">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="7">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="7">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="7">
+        <v>4700</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="7">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="7">
         <v>650</v>
       </c>
     </row>
@@ -578,72 +681,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>9</v>
+      <c r="A1" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
+      <c r="A2" s="4"/>
     </row>
     <row r="3" spans="1:1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>10</v>
+      <c r="A3" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="5"/>
+      <c r="A4" s="4"/>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>11</v>
+      <c r="A5" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>12</v>
+      <c r="A6" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>13</v>
+      <c r="A7" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>14</v>
+      <c r="A8" s="5" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>15</v>
+      <c r="A9" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>16</v>
+      <c r="A10" s="5" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
+      <c r="A11" s="4"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>17</v>
+      <c r="A12" s="6" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>18</v>
+      <c r="A13" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>19</v>
+      <c r="A14" s="5" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>20</v>
+      <c r="A15" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>